<commit_message>
rules and op dir path
</commit_message>
<xml_diff>
--- a/docs/mci_cog_igm_rules_dcc.xlsx
+++ b/docs/mci_cog_igm_rules_dcc.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bullenca/Work/CCDIDC/CCDIDC-1950/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bullenca/Work/Repos/ChildhoodCancerDataInitiative-Prefect_Pipeline/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{176B4ED1-C734-C24F-9A84-1C3AF7176F66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67695254-1F30-9848-A275-937909D91686}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17820" xr2:uid="{9DC53540-95BC-6744-B593-4545FF261AF8}"/>
+    <workbookView xWindow="20320" yWindow="-19520" windowWidth="30240" windowHeight="17820" xr2:uid="{9DC53540-95BC-6744-B593-4545FF261AF8}"/>
   </bookViews>
   <sheets>
     <sheet name="cog_rules" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2053" uniqueCount="223">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2064" uniqueCount="223">
   <si>
     <t>source</t>
   </si>
@@ -2157,8 +2157,8 @@
       <c r="I24" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="J24">
-        <v>-999</v>
+      <c r="J24" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.2">
@@ -2508,8 +2508,8 @@
       <c r="I39" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="J39">
-        <v>-999</v>
+      <c r="J39" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.2">
@@ -2850,8 +2850,8 @@
       <c r="I54" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="J54">
-        <v>-999</v>
+      <c r="J54" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.2">
@@ -3201,8 +3201,8 @@
       <c r="I69" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="J69">
-        <v>-999</v>
+      <c r="J69" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="70" spans="1:10" x14ac:dyDescent="0.2">
@@ -3549,8 +3549,8 @@
       <c r="I84" t="s">
         <v>85</v>
       </c>
-      <c r="J84">
-        <v>-999</v>
+      <c r="J84" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="85" spans="1:10" x14ac:dyDescent="0.2">
@@ -3796,6 +3796,9 @@
       <c r="F95" t="s">
         <v>74</v>
       </c>
+      <c r="G95" t="s">
+        <v>47</v>
+      </c>
       <c r="H95" t="s">
         <v>73</v>
       </c>
@@ -3897,8 +3900,8 @@
       <c r="I99" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="J99">
-        <v>-999</v>
+      <c r="J99" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="100" spans="1:10" x14ac:dyDescent="0.2">
@@ -4254,8 +4257,8 @@
       <c r="I114" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="J114">
-        <v>-999</v>
+      <c r="J114" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="115" spans="1:10" x14ac:dyDescent="0.2">
@@ -4605,8 +4608,8 @@
       <c r="I129" t="s">
         <v>85</v>
       </c>
-      <c r="J129">
-        <v>-999</v>
+      <c r="J129" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="130" spans="1:10" x14ac:dyDescent="0.2">
@@ -4962,8 +4965,8 @@
       <c r="I144" t="s">
         <v>85</v>
       </c>
-      <c r="J144">
-        <v>-999</v>
+      <c r="J144" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="145" spans="1:10" x14ac:dyDescent="0.2">
@@ -5316,8 +5319,8 @@
       <c r="I159" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="J159">
-        <v>-999</v>
+      <c r="J159" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="160" spans="1:10" x14ac:dyDescent="0.2">

</xml_diff>